<commit_message>
Perbarui data SE2026 23/08/2026 20:24:35,89
</commit_message>
<xml_diff>
--- a/data/Export_Monitoring_SLS_Kabupaten_Kota.xlsx
+++ b/data/Export_Monitoring_SLS_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
   <si>
     <t>MONITORING SLS</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 23 Agu 2026, 12.04 | Dicetak: 23 Agu 2026, 12.52</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 23 Agu 2026, 18.04 | Dicetak: 23 Agu 2026, 20.21</t>
   </si>
   <si>
     <t>Kode</t>
@@ -55,7 +55,7 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>7,59</t>
+    <t>7,56</t>
   </si>
   <si>
     <t>1801</t>
@@ -82,7 +82,7 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>3,16</t>
+    <t>3,22</t>
   </si>
   <si>
     <t>1804</t>
@@ -91,7 +91,7 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>2,08</t>
+    <t>2,12</t>
   </si>
   <si>
     <t>1805</t>
@@ -100,7 +100,7 @@
     <t>LAMPUNG TENGAH</t>
   </si>
   <si>
-    <t>2,59</t>
+    <t>2,56</t>
   </si>
   <si>
     <t>1806</t>
@@ -127,7 +127,7 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>15,74</t>
+    <t>15,77</t>
   </si>
   <si>
     <t>1809</t>
@@ -136,7 +136,7 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>20,27</t>
+    <t>20,23</t>
   </si>
   <si>
     <t>1810</t>
@@ -154,7 +154,7 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>25,25</t>
+    <t>24,36</t>
   </si>
   <si>
     <t>1812</t>
@@ -172,7 +172,7 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>28,06</t>
+    <t>27,41</t>
   </si>
   <si>
     <t>1871</t>
@@ -181,13 +181,16 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>0,52</t>
+    <t>0,58</t>
   </si>
   <si>
     <t>1872</t>
   </si>
   <si>
     <t>METRO</t>
+  </si>
+  <si>
+    <t>3,27</t>
   </si>
   <si>
     <t/>
@@ -756,7 +759,7 @@
         <v>49386</v>
       </c>
       <c r="D6" s="6">
-        <v>3748</v>
+        <v>3734</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>14</v>
@@ -807,7 +810,7 @@
         <v>5816</v>
       </c>
       <c r="D9" s="9">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>23</v>
@@ -824,7 +827,7 @@
         <v>6824</v>
       </c>
       <c r="D10" s="9">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>26</v>
@@ -841,7 +844,7 @@
         <v>8607</v>
       </c>
       <c r="D11" s="9">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>29</v>
@@ -892,7 +895,7 @@
         <v>3900</v>
       </c>
       <c r="D14" s="9">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>38</v>
@@ -909,7 +912,7 @@
         <v>2753</v>
       </c>
       <c r="D15" s="9">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>41</v>
@@ -943,7 +946,7 @@
         <v>1802</v>
       </c>
       <c r="D17" s="9">
-        <v>455</v>
+        <v>439</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>47</v>
@@ -977,7 +980,7 @@
         <v>613</v>
       </c>
       <c r="D19" s="9">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>53</v>
@@ -994,7 +997,7 @@
         <v>3432</v>
       </c>
       <c r="D20" s="9">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>56</v>
@@ -1011,24 +1014,24 @@
         <v>855</v>
       </c>
       <c r="D21" s="9">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C22" s="12">
         <v>49386</v>
       </c>
       <c r="D22" s="12">
-        <v>3748</v>
+        <v>3734</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 24/08/2026 21:19:32,52
</commit_message>
<xml_diff>
--- a/data/Export_Monitoring_SLS_Kabupaten_Kota.xlsx
+++ b/data/Export_Monitoring_SLS_Kabupaten_Kota.xlsx
@@ -16,7 +16,7 @@
     <t>MONITORING SLS</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 24 Agu 2026, 06.04 | Dicetak: 24 Agu 2026, 07.46</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 24 Agu 2026, 18.04 | Dicetak: 24 Agu 2026, 21.08</t>
   </si>
   <si>
     <t>Kode</t>
@@ -55,7 +55,7 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>7,65</t>
+    <t>7,8</t>
   </si>
   <si>
     <t>1801</t>
@@ -82,7 +82,7 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>3,35</t>
+    <t>3,51</t>
   </si>
   <si>
     <t>1804</t>
@@ -91,7 +91,7 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>2,1</t>
+    <t>2,15</t>
   </si>
   <si>
     <t>1805</t>
@@ -100,7 +100,7 @@
     <t>LAMPUNG TENGAH</t>
   </si>
   <si>
-    <t>2,58</t>
+    <t>2,6</t>
   </si>
   <si>
     <t>1806</t>
@@ -109,7 +109,7 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>16,06</t>
+    <t>16,01</t>
   </si>
   <si>
     <t>1807</t>
@@ -127,7 +127,7 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>16,05</t>
+    <t>16,03</t>
   </si>
   <si>
     <t>1809</t>
@@ -136,7 +136,7 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>20,34</t>
+    <t>21,76</t>
   </si>
   <si>
     <t>1810</t>
@@ -145,7 +145,7 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>11,9</t>
+    <t>12,15</t>
   </si>
   <si>
     <t>1811</t>
@@ -154,7 +154,7 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>23,97</t>
+    <t>23,81</t>
   </si>
   <si>
     <t>1812</t>
@@ -163,7 +163,7 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>19,68</t>
+    <t>20,85</t>
   </si>
   <si>
     <t>1813</t>
@@ -172,7 +172,7 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>26,43</t>
+    <t>24,63</t>
   </si>
   <si>
     <t>1871</t>
@@ -181,7 +181,7 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>0,67</t>
+    <t>0,73</t>
   </si>
   <si>
     <t>1872</t>
@@ -190,7 +190,7 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>3,27</t>
+    <t>3,04</t>
   </si>
   <si>
     <t/>
@@ -759,7 +759,7 @@
         <v>49386</v>
       </c>
       <c r="D6" s="6">
-        <v>3780</v>
+        <v>3850</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>14</v>
@@ -810,7 +810,7 @@
         <v>5816</v>
       </c>
       <c r="D9" s="9">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>23</v>
@@ -827,7 +827,7 @@
         <v>6824</v>
       </c>
       <c r="D10" s="9">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>26</v>
@@ -844,7 +844,7 @@
         <v>8607</v>
       </c>
       <c r="D11" s="9">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>29</v>
@@ -861,7 +861,7 @@
         <v>4022</v>
       </c>
       <c r="D12" s="9">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>32</v>
@@ -895,7 +895,7 @@
         <v>3900</v>
       </c>
       <c r="D14" s="9">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>38</v>
@@ -912,7 +912,7 @@
         <v>2753</v>
       </c>
       <c r="D15" s="9">
-        <v>560</v>
+        <v>599</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>41</v>
@@ -929,7 +929,7 @@
         <v>1605</v>
       </c>
       <c r="D16" s="9">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>44</v>
@@ -946,7 +946,7 @@
         <v>1802</v>
       </c>
       <c r="D17" s="9">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>47</v>
@@ -963,7 +963,7 @@
         <v>2485</v>
       </c>
       <c r="D18" s="9">
-        <v>489</v>
+        <v>518</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>50</v>
@@ -980,7 +980,7 @@
         <v>613</v>
       </c>
       <c r="D19" s="9">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>53</v>
@@ -997,7 +997,7 @@
         <v>3432</v>
       </c>
       <c r="D20" s="9">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>56</v>
@@ -1014,7 +1014,7 @@
         <v>855</v>
       </c>
       <c r="D21" s="9">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>59</v>
@@ -1031,7 +1031,7 @@
         <v>49386</v>
       </c>
       <c r="D22" s="12">
-        <v>3780</v>
+        <v>3850</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>14</v>

</xml_diff>